<commit_message>
Corrige processamento de beneficios
</commit_message>
<xml_diff>
--- a/projeto/centros_de_custo.xlsx
+++ b/projeto/centros_de_custo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\projeto_atendimento\NIBO WEB API\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bened\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C54375FB-C8B9-425F-AA57-D4BB6FEE0E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0925EB84-3FF1-49E6-8255-B5A349222C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13335" xr2:uid="{1458C256-756D-4BF1-B610-992632ACD84E}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{1458C256-756D-4BF1-B610-992632ACD84E}"/>
   </bookViews>
   <sheets>
     <sheet name="Centro de Custo" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="262">
   <si>
     <t>d7f01dc1-d4cf-4158-ae39-003526a50440</t>
   </si>
@@ -816,6 +816,12 @@
   </si>
   <si>
     <t>FENDI</t>
+  </si>
+  <si>
+    <t>e155241e-3fba-4ff8-9dcb-b7e792eb03b1</t>
+  </si>
+  <si>
+    <t>NEW ERA</t>
   </si>
 </sst>
 </file>
@@ -1195,14 +1201,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{163D22BB-575F-489C-9799-F85DA17AF1ED}">
-  <dimension ref="A1:C130"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C131"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="45.9296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>182</v>
       </c>
@@ -1213,7 +1219,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>418</v>
       </c>
@@ -1224,7 +1230,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>80</v>
       </c>
@@ -1235,7 +1241,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>4</v>
       </c>
@@ -1246,7 +1252,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>463</v>
       </c>
@@ -1257,7 +1263,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>223</v>
       </c>
@@ -1268,7 +1274,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>468</v>
       </c>
@@ -1279,7 +1285,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>462</v>
       </c>
@@ -1290,7 +1296,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>427</v>
       </c>
@@ -1301,7 +1307,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>244</v>
       </c>
@@ -1312,7 +1318,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>421</v>
       </c>
@@ -1323,7 +1329,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>284</v>
       </c>
@@ -1334,7 +1340,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>294</v>
       </c>
@@ -1345,7 +1351,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>405</v>
       </c>
@@ -1356,7 +1362,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>389</v>
       </c>
@@ -1367,7 +1373,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>410</v>
       </c>
@@ -1378,7 +1384,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>440</v>
       </c>
@@ -1389,7 +1395,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>163</v>
       </c>
@@ -1400,7 +1406,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>471</v>
       </c>
@@ -1411,7 +1417,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>451</v>
       </c>
@@ -1422,7 +1428,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>293</v>
       </c>
@@ -1433,7 +1439,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>261</v>
       </c>
@@ -1444,7 +1450,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>245</v>
       </c>
@@ -1455,7 +1461,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>353</v>
       </c>
@@ -1466,7 +1472,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>441</v>
       </c>
@@ -1477,7 +1483,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>336</v>
       </c>
@@ -1488,7 +1494,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>14</v>
       </c>
@@ -1499,7 +1505,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>401</v>
       </c>
@@ -1510,7 +1516,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>376</v>
       </c>
@@ -1521,7 +1527,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>16</v>
       </c>
@@ -1532,7 +1538,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31">
         <v>189</v>
       </c>
@@ -1543,7 +1549,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32">
         <v>447</v>
       </c>
@@ -1554,7 +1560,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33">
         <v>323</v>
       </c>
@@ -1565,7 +1571,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34">
         <v>236</v>
       </c>
@@ -1576,7 +1582,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>237</v>
       </c>
@@ -1587,7 +1593,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>235</v>
       </c>
@@ -1598,7 +1604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37">
         <v>335</v>
       </c>
@@ -1609,7 +1615,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38">
         <v>253</v>
       </c>
@@ -1620,7 +1626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>340</v>
       </c>
@@ -1631,7 +1637,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>342</v>
       </c>
@@ -1642,7 +1648,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>64</v>
       </c>
@@ -1653,7 +1659,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>211</v>
       </c>
@@ -1664,7 +1670,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A43">
         <v>445</v>
       </c>
@@ -1675,7 +1681,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A44">
         <v>446</v>
       </c>
@@ -1686,7 +1692,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A45">
         <v>412</v>
       </c>
@@ -1697,7 +1703,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A46">
         <v>346</v>
       </c>
@@ -1708,7 +1714,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A47">
         <v>105</v>
       </c>
@@ -1719,7 +1725,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>390</v>
       </c>
@@ -1730,7 +1736,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A49">
         <v>411</v>
       </c>
@@ -1741,7 +1747,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>450</v>
       </c>
@@ -1752,7 +1758,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A51">
         <v>312</v>
       </c>
@@ -1763,7 +1769,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A52">
         <v>304</v>
       </c>
@@ -1774,7 +1780,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A53">
         <v>228</v>
       </c>
@@ -1785,7 +1791,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A54">
         <v>241</v>
       </c>
@@ -1796,7 +1802,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A55">
         <v>234</v>
       </c>
@@ -1807,7 +1813,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A56">
         <v>233</v>
       </c>
@@ -1818,7 +1824,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A57">
         <v>362</v>
       </c>
@@ -1829,7 +1835,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A58">
         <v>370</v>
       </c>
@@ -1840,7 +1846,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A59">
         <v>217</v>
       </c>
@@ -1851,7 +1857,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A60">
         <v>255</v>
       </c>
@@ -1862,7 +1868,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A61">
         <v>444</v>
       </c>
@@ -1873,7 +1879,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A62">
         <v>382</v>
       </c>
@@ -1884,7 +1890,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A63">
         <v>263</v>
       </c>
@@ -1895,7 +1901,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A64">
         <v>363</v>
       </c>
@@ -1906,7 +1912,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A65">
         <v>330</v>
       </c>
@@ -1917,7 +1923,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A66">
         <v>160</v>
       </c>
@@ -1928,7 +1934,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A67">
         <v>379</v>
       </c>
@@ -1939,7 +1945,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A68">
         <v>374</v>
       </c>
@@ -1950,7 +1956,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A69">
         <v>474</v>
       </c>
@@ -1961,7 +1967,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A70">
         <v>470</v>
       </c>
@@ -1972,7 +1978,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A71">
         <v>171</v>
       </c>
@@ -1983,7 +1989,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A72">
         <v>345</v>
       </c>
@@ -1994,7 +2000,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A73">
         <v>465</v>
       </c>
@@ -2005,7 +2011,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A74">
         <v>352</v>
       </c>
@@ -2016,7 +2022,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A75">
         <v>442</v>
       </c>
@@ -2027,7 +2033,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A76">
         <v>423</v>
       </c>
@@ -2038,7 +2044,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A77">
         <v>157</v>
       </c>
@@ -2049,7 +2055,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A78">
         <v>443</v>
       </c>
@@ -2060,7 +2066,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A79">
         <v>360</v>
       </c>
@@ -2071,7 +2077,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A80">
         <v>402</v>
       </c>
@@ -2082,7 +2088,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A81">
         <v>321</v>
       </c>
@@ -2093,7 +2099,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A82">
         <v>358</v>
       </c>
@@ -2104,7 +2110,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A83">
         <v>359</v>
       </c>
@@ -2115,7 +2121,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A84">
         <v>197</v>
       </c>
@@ -2126,7 +2132,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A85">
         <v>425</v>
       </c>
@@ -2137,7 +2143,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A86">
         <v>338</v>
       </c>
@@ -2148,7 +2154,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A87">
         <v>469</v>
       </c>
@@ -2159,7 +2165,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A88">
         <v>218</v>
       </c>
@@ -2170,7 +2176,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A89">
         <v>194</v>
       </c>
@@ -2181,7 +2187,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A90">
         <v>158</v>
       </c>
@@ -2192,7 +2198,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A91">
         <v>226</v>
       </c>
@@ -2203,7 +2209,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A92">
         <v>202</v>
       </c>
@@ -2214,7 +2220,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A93">
         <v>439</v>
       </c>
@@ -2225,7 +2231,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A94">
         <v>291</v>
       </c>
@@ -2236,7 +2242,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A95">
         <v>467</v>
       </c>
@@ -2247,7 +2253,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A96">
         <v>384</v>
       </c>
@@ -2258,7 +2264,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A97">
         <v>383</v>
       </c>
@@ -2269,7 +2275,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A98">
         <v>246</v>
       </c>
@@ -2280,7 +2286,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A99">
         <v>256</v>
       </c>
@@ -2291,7 +2297,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A100">
         <v>273</v>
       </c>
@@ -2302,7 +2308,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A101">
         <v>407</v>
       </c>
@@ -2313,7 +2319,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A102">
         <v>449</v>
       </c>
@@ -2324,7 +2330,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A103">
         <v>464</v>
       </c>
@@ -2335,7 +2341,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A104">
         <v>258</v>
       </c>
@@ -2346,7 +2352,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A105">
         <v>317</v>
       </c>
@@ -2357,7 +2363,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A106">
         <v>324</v>
       </c>
@@ -2368,7 +2374,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A107">
         <v>341</v>
       </c>
@@ -2379,7 +2385,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A108">
         <v>308</v>
       </c>
@@ -2390,7 +2396,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A109">
         <v>380</v>
       </c>
@@ -2401,7 +2407,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A110">
         <v>466</v>
       </c>
@@ -2412,7 +2418,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A111">
         <v>103</v>
       </c>
@@ -2423,7 +2429,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A112">
         <v>453</v>
       </c>
@@ -2434,7 +2440,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A113">
         <v>475</v>
       </c>
@@ -2445,7 +2451,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A114">
         <v>7</v>
       </c>
@@ -2456,7 +2462,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A115">
         <v>454</v>
       </c>
@@ -2467,7 +2473,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A116">
         <v>377</v>
       </c>
@@ -2478,7 +2484,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A117">
         <v>295</v>
       </c>
@@ -2489,7 +2495,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A118">
         <v>350</v>
       </c>
@@ -2500,7 +2506,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A119">
         <v>152</v>
       </c>
@@ -2511,7 +2517,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A120">
         <v>413</v>
       </c>
@@ -2522,7 +2528,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A121">
         <v>473</v>
       </c>
@@ -2533,7 +2539,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A122">
         <v>381</v>
       </c>
@@ -2544,7 +2550,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A123">
         <v>248</v>
       </c>
@@ -2555,7 +2561,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A124">
         <v>406</v>
       </c>
@@ -2566,7 +2572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A125">
         <v>487</v>
       </c>
@@ -2577,7 +2583,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A126">
         <v>478</v>
       </c>
@@ -2588,7 +2594,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A127">
         <v>482</v>
       </c>
@@ -2599,7 +2605,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A128">
         <v>193</v>
       </c>
@@ -2610,7 +2616,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A129">
         <v>483</v>
       </c>
@@ -2621,7 +2627,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A130">
         <v>209</v>
       </c>
@@ -2632,7 +2638,19 @@
         <v>258</v>
       </c>
     </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A131">
+        <v>489</v>
+      </c>
+      <c r="B131" t="s">
+        <v>261</v>
+      </c>
+      <c r="C131" t="s">
+        <v>260</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>